<commit_message>
fix: nombres únicos en el padrón de ejemplo
Las filas con DNI 50000042-50000060 repetían los nombres de las filas
50000022-50000040; se renombraron manteniendo DNI, género y tipo de
banca. El test ahora verifica que no haya nombre+apellido repetidos.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/example-ppc.xlsx
+++ b/example-ppc.xlsx
@@ -1,17 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-  <workbookPr/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xml:space="preserve">
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+  <workbookPr codeName="ThisWorkbook"/>
+  <bookViews>
+    <workbookView activeTab="0" autoFilterDateGrouping="true" firstSheet="0" minimized="false" showHorizontalScroll="true" showSheetTabs="true" showVerticalScroll="true" tabRatio="600" visibility="visible"/>
+  </bookViews>
   <sheets>
-    <sheet state="visible" name="Hoja 1" sheetId="1" r:id="rId5"/>
+    <sheet name="Hoja 1" sheetId="1" r:id="rId4"/>
   </sheets>
   <definedNames/>
-  <calcPr/>
+  <calcPr calcId="999999" calcMode="auto" calcCompleted="1" fullCalcOnLoad="0" forceFullCalc="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="185" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="87">
   <si>
     <t>Nombre</t>
   </si>
@@ -160,37 +164,173 @@
   </si>
   <si>
     <t>Rodriguez</t>
+  </si>
+  <si>
+    <t>Ramiro</t>
+  </si>
+  <si>
+    <t>Ledesma</t>
+  </si>
+  <si>
+    <t>Paula</t>
+  </si>
+  <si>
+    <t>Giménez</t>
+  </si>
+  <si>
+    <t>Esteban</t>
+  </si>
+  <si>
+    <t>Núñez</t>
+  </si>
+  <si>
+    <t>Rocío</t>
+  </si>
+  <si>
+    <t>Cabrera</t>
+  </si>
+  <si>
+    <t>Gonzalo</t>
+  </si>
+  <si>
+    <t>Duarte</t>
+  </si>
+  <si>
+    <t>Milagros</t>
+  </si>
+  <si>
+    <t>Vera</t>
+  </si>
+  <si>
+    <t>Facundo</t>
+  </si>
+  <si>
+    <t>Ríos</t>
+  </si>
+  <si>
+    <t>Antonella</t>
+  </si>
+  <si>
+    <t>Sosa</t>
+  </si>
+  <si>
+    <t>Alex</t>
+  </si>
+  <si>
+    <t>Aguirre</t>
+  </si>
+  <si>
+    <t>Daniela</t>
+  </si>
+  <si>
+    <t>Ferreyra</t>
+  </si>
+  <si>
+    <t>Marcela</t>
+  </si>
+  <si>
+    <t>Ojeda</t>
+  </si>
+  <si>
+    <t>Rubén</t>
+  </si>
+  <si>
+    <t>Villalba</t>
+  </si>
+  <si>
+    <t>Maximiliano</t>
+  </si>
+  <si>
+    <t>Correa</t>
+  </si>
+  <si>
+    <t>Brenda</t>
+  </si>
+  <si>
+    <t>Escobar</t>
+  </si>
+  <si>
+    <t>Leandro</t>
+  </si>
+  <si>
+    <t>Paredes</t>
+  </si>
+  <si>
+    <t>Melina</t>
+  </si>
+  <si>
+    <t>Barrios</t>
+  </si>
+  <si>
+    <t>Cristian</t>
+  </si>
+  <si>
+    <t>Godoy</t>
+  </si>
+  <si>
+    <t>Iván</t>
+  </si>
+  <si>
+    <t>Maidana</t>
+  </si>
+  <si>
+    <t>Carolina</t>
+  </si>
+  <si>
+    <t>Olivera</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xml:space="preserve">
+  <numFmts count="0"/>
   <fonts count="5">
     <font>
-      <sz val="10.0"/>
+      <b val="0"/>
+      <i val="0"/>
+      <strike val="0"/>
+      <u val="none"/>
+      <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <color theme="1"/>
+      <b val="1"/>
+      <i val="0"/>
+      <strike val="0"/>
+      <u val="none"/>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="11.0"/>
-      <color theme="1"/>
+      <b val="0"/>
+      <i val="0"/>
+      <strike val="0"/>
+      <u val="none"/>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
       <name val="Aptos Narrow"/>
     </font>
     <font>
-      <sz val="11.0"/>
-      <color theme="1"/>
+      <b val="0"/>
+      <i val="0"/>
+      <strike val="0"/>
+      <u val="none"/>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
       <name val="Arial"/>
     </font>
     <font>
-      <color theme="1"/>
+      <b val="0"/>
+      <i val="0"/>
+      <strike val="0"/>
+      <u val="none"/>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
@@ -200,7 +340,7 @@
       <patternFill patternType="none"/>
     </fill>
     <fill>
-      <patternFill patternType="lightGray"/>
+      <patternFill patternType="gray125"/>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -210,7 +350,13 @@
     </fill>
   </fills>
   <borders count="2">
-    <border/>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
     <border>
       <left style="thin">
         <color rgb="FF000000"/>
@@ -224,72 +370,36 @@
       <bottom style="thin">
         <color rgb="FF000000"/>
       </bottom>
+      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="7">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="0" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0"/>
+    <xf xfId="0" fontId="1" numFmtId="0" fillId="0" borderId="1" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" shrinkToFit="false"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    <xf xfId="0" fontId="2" numFmtId="0" fillId="0" borderId="1" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" shrinkToFit="false"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="right" vertical="bottom"/>
+    <xf xfId="0" fontId="2" numFmtId="0" fillId="2" borderId="1" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" shrinkToFit="false"/>
     </xf>
-    <xf borderId="1" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="right" vertical="bottom"/>
+    <xf xfId="0" fontId="2" numFmtId="0" fillId="0" borderId="1" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" shrinkToFit="false"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="right" vertical="bottom"/>
+    <xf xfId="0" fontId="3" numFmtId="0" fillId="2" borderId="1" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" shrinkToFit="false"/>
     </xf>
-    <xf borderId="1" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="right" readingOrder="0" vertical="bottom"/>
-    </xf>
-    <xf borderId="1" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
+    <xf xfId="0" fontId="4" numFmtId="0" fillId="0" borderId="1" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle xfId="0" name="Normal" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="3">
-    <dxf>
-      <font/>
-      <fill>
-        <patternFill patternType="none"/>
-      </fill>
-      <border/>
-    </dxf>
-    <dxf>
-      <font/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFD8D8D8"/>
-          <bgColor rgb="FFD8D8D8"/>
-        </patternFill>
-      </fill>
-      <border/>
-    </dxf>
-    <dxf>
-      <font/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="0"/>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-      <border/>
-    </dxf>
-  </dxfs>
-  <tableStyles count="1">
-    <tableStyle count="2" pivot="0" name="Hoja 1-style">
-      <tableStyleElement dxfId="1" type="firstRowStripe"/>
-      <tableStyleElement dxfId="2" type="secondRowStripe"/>
-    </tableStyle>
-  </tableStyles>
+  <dxfs count="0"/>
+  <tableStyles defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotTableStyle1"/>
 </styleSheet>
 </file>
 
@@ -297,28 +407,24 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
 </file>
 
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<x18tc:personList xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments"/>
-</file>
-
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" headerRowCount="0" ref="D2:D61" displayName="Table_1" name="Table_1" id="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xml:space="preserve" id="1" name="Table1" displayName="Table_1" ref="D2:D61" headerRowCount="0" totalsRowCount="0">
   <tableColumns count="1">
-    <tableColumn name="Column1" id="1"/>
+    <tableColumn id="1" name="Column1"/>
   </tableColumns>
-  <tableStyleInfo name="Hoja 1-style" showColumnStripes="0" showFirstColumn="1" showLastColumn="1" showRowStripes="1"/>
+  <tableStyleInfo name="Hoja 1-style" showFirstColumn="1" showLastColumn="1" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheets">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Sheets">
       <a:dk1>
-        <a:srgbClr val="000000"/>
+        <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:srgbClr val="FFFFFF"/>
+        <a:sysClr val="window" lastClr="FFFFFF"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="000000"/>
@@ -372,146 +478,178 @@
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:lumMod val="110000"/>
-                <a:satMod val="105000"/>
-                <a:tint val="67000"/>
+                <a:tint val="50000"/>
+                <a:satMod val="300000"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="50000">
+            <a:gs pos="35000">
               <a:schemeClr val="phClr">
-                <a:lumMod val="105000"/>
-                <a:satMod val="103000"/>
-                <a:tint val="73000"/>
+                <a:tint val="37000"/>
+                <a:satMod val="300000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:lumMod val="105000"/>
-                <a:satMod val="109000"/>
-                <a:tint val="81000"/>
+                <a:tint val="15000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:lin ang="16200000" scaled="1"/>
         </a:gradFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:satMod val="103000"/>
-                <a:lumMod val="102000"/>
-                <a:tint val="94000"/>
+                <a:shade val="51000"/>
+                <a:satMod val="130000"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="50000">
+            <a:gs pos="80000">
               <a:schemeClr val="phClr">
-                <a:satMod val="110000"/>
-                <a:lumMod val="100000"/>
-                <a:shade val="100000"/>
+                <a:shade val="93000"/>
+                <a:satMod val="130000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:lumMod val="99000"/>
-                <a:satMod val="120000"/>
-                <a:shade val="78000"/>
+                <a:shade val="94000"/>
+                <a:satMod val="135000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:lin ang="16200000" scaled="0"/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr">
+              <a:shade val="95000"/>
+              <a:satMod val="105000"/>
+            </a:schemeClr>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
         </a:ln>
-        <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
-        </a:ln>
-        <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
         </a:ln>
       </a:lnStyleLst>
       <a:effectStyleLst>
         <a:effectStyle>
-          <a:effectLst/>
-        </a:effectStyle>
-        <a:effectStyle>
-          <a:effectLst/>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="20000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="38000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
-                <a:alpha val="63000"/>
+                <a:alpha val="35000"/>
               </a:srgbClr>
             </a:outerShdw>
           </a:effectLst>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+          <a:scene3d>
+            <a:camera prst="orthographicFront">
+              <a:rot lat="0" lon="0" rev="0"/>
+            </a:camera>
+            <a:lightRig rig="threePt" dir="t">
+              <a:rot lat="0" lon="0" rev="1200000"/>
+            </a:lightRig>
+          </a:scene3d>
+          <a:sp3d>
+            <a:bevelT w="63500" h="25400"/>
+          </a:sp3d>
         </a:effectStyle>
       </a:effectStyleLst>
       <a:bgFillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
-        <a:solidFill>
-          <a:schemeClr val="phClr">
-            <a:tint val="95000"/>
-            <a:satMod val="170000"/>
-          </a:schemeClr>
-        </a:solidFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:tint val="93000"/>
-                <a:satMod val="150000"/>
-                <a:shade val="98000"/>
-                <a:lumMod val="102000"/>
+                <a:tint val="40000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="50000">
+            <a:gs pos="40000">
               <a:schemeClr val="phClr">
-                <a:tint val="98000"/>
-                <a:satMod val="130000"/>
-                <a:shade val="90000"/>
-                <a:lumMod val="103000"/>
+                <a:tint val="45000"/>
+                <a:shade val="99000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:shade val="63000"/>
-                <a:satMod val="120000"/>
+                <a:shade val="20000"/>
+                <a:satMod val="255000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
+          </a:path>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="80000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="30000"/>
+                <a:satMod val="200000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
+          </a:path>
         </a:gradFill>
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xml:space="preserve" mc:Ignorable="x14ac">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <dimension ref="A1:E61"/>
+  <sheetFormatPr customHeight="true" defaultRowHeight="15.75" defaultColWidth="12.63" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:5">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -528,7 +666,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" spans="1:5">
       <c r="A2" s="2" t="s">
         <v>5</v>
       </c>
@@ -536,7 +674,7 @@
         <v>6</v>
       </c>
       <c r="C2" s="2">
-        <v>5.0000001E7</v>
+        <v>50000001.0</v>
       </c>
       <c r="D2" s="3" t="s">
         <v>7</v>
@@ -545,7 +683,7 @@
         <v>2.0</v>
       </c>
     </row>
-    <row r="3">
+    <row r="3" spans="1:5">
       <c r="A3" s="2" t="s">
         <v>8</v>
       </c>
@@ -553,7 +691,7 @@
         <v>9</v>
       </c>
       <c r="C3" s="2">
-        <f t="shared" ref="C3:C61" si="1">50000000+ROW(A1)+1</f>
+        <f>50000000+ROW(A1)+1</f>
         <v>50000002</v>
       </c>
       <c r="D3" s="3" t="s">
@@ -563,7 +701,7 @@
         <v>2.0</v>
       </c>
     </row>
-    <row r="4">
+    <row r="4" spans="1:5">
       <c r="A4" s="2" t="s">
         <v>10</v>
       </c>
@@ -571,7 +709,7 @@
         <v>11</v>
       </c>
       <c r="C4" s="2">
-        <f t="shared" si="1"/>
+        <f>50000000+ROW(A2)+1</f>
         <v>50000003</v>
       </c>
       <c r="D4" s="3" t="s">
@@ -581,7 +719,7 @@
         <v>4.0</v>
       </c>
     </row>
-    <row r="5">
+    <row r="5" spans="1:5">
       <c r="A5" s="2" t="s">
         <v>13</v>
       </c>
@@ -589,7 +727,7 @@
         <v>14</v>
       </c>
       <c r="C5" s="2">
-        <f t="shared" si="1"/>
+        <f>50000000+ROW(A3)+1</f>
         <v>50000004</v>
       </c>
       <c r="D5" s="3" t="s">
@@ -599,7 +737,7 @@
         <v>3.0</v>
       </c>
     </row>
-    <row r="6">
+    <row r="6" spans="1:5">
       <c r="A6" s="2" t="s">
         <v>15</v>
       </c>
@@ -607,7 +745,7 @@
         <v>16</v>
       </c>
       <c r="C6" s="2">
-        <f t="shared" si="1"/>
+        <f>50000000+ROW(A4)+1</f>
         <v>50000005</v>
       </c>
       <c r="D6" s="3" t="s">
@@ -617,7 +755,7 @@
         <v>3.0</v>
       </c>
     </row>
-    <row r="7">
+    <row r="7" spans="1:5">
       <c r="A7" s="2" t="s">
         <v>17</v>
       </c>
@@ -625,7 +763,7 @@
         <v>18</v>
       </c>
       <c r="C7" s="2">
-        <f t="shared" si="1"/>
+        <f>50000000+ROW(A5)+1</f>
         <v>50000006</v>
       </c>
       <c r="D7" s="3" t="s">
@@ -635,7 +773,7 @@
         <v>4.0</v>
       </c>
     </row>
-    <row r="8">
+    <row r="8" spans="1:5">
       <c r="A8" s="2" t="s">
         <v>19</v>
       </c>
@@ -643,7 +781,7 @@
         <v>20</v>
       </c>
       <c r="C8" s="2">
-        <f t="shared" si="1"/>
+        <f>50000000+ROW(A6)+1</f>
         <v>50000007</v>
       </c>
       <c r="D8" s="3" t="s">
@@ -653,7 +791,7 @@
         <v>4.0</v>
       </c>
     </row>
-    <row r="9">
+    <row r="9" spans="1:5">
       <c r="A9" s="2" t="s">
         <v>21</v>
       </c>
@@ -661,7 +799,7 @@
         <v>22</v>
       </c>
       <c r="C9" s="2">
-        <f t="shared" si="1"/>
+        <f>50000000+ROW(A7)+1</f>
         <v>50000008</v>
       </c>
       <c r="D9" s="3" t="s">
@@ -671,7 +809,7 @@
         <v>4.0</v>
       </c>
     </row>
-    <row r="10">
+    <row r="10" spans="1:5">
       <c r="A10" s="2" t="s">
         <v>23</v>
       </c>
@@ -679,7 +817,7 @@
         <v>24</v>
       </c>
       <c r="C10" s="2">
-        <f t="shared" si="1"/>
+        <f>50000000+ROW(A8)+1</f>
         <v>50000009</v>
       </c>
       <c r="D10" s="3" t="s">
@@ -689,7 +827,7 @@
         <v>4.0</v>
       </c>
     </row>
-    <row r="11">
+    <row r="11" spans="1:5">
       <c r="A11" s="2" t="s">
         <v>25</v>
       </c>
@@ -697,7 +835,7 @@
         <v>26</v>
       </c>
       <c r="C11" s="2">
-        <f t="shared" si="1"/>
+        <f>50000000+ROW(A9)+1</f>
         <v>50000010</v>
       </c>
       <c r="D11" s="5" t="s">
@@ -707,7 +845,7 @@
         <v>3.0</v>
       </c>
     </row>
-    <row r="12">
+    <row r="12" spans="1:5">
       <c r="A12" s="2" t="s">
         <v>28</v>
       </c>
@@ -715,7 +853,7 @@
         <v>29</v>
       </c>
       <c r="C12" s="2">
-        <f t="shared" si="1"/>
+        <f>50000000+ROW(A10)+1</f>
         <v>50000011</v>
       </c>
       <c r="D12" s="5" t="s">
@@ -725,7 +863,7 @@
         <v>3.0</v>
       </c>
     </row>
-    <row r="13">
+    <row r="13" spans="1:5">
       <c r="A13" s="2" t="s">
         <v>30</v>
       </c>
@@ -733,7 +871,7 @@
         <v>31</v>
       </c>
       <c r="C13" s="2">
-        <f t="shared" si="1"/>
+        <f>50000000+ROW(A11)+1</f>
         <v>50000012</v>
       </c>
       <c r="D13" s="3" t="s">
@@ -743,7 +881,7 @@
         <v>2.0</v>
       </c>
     </row>
-    <row r="14">
+    <row r="14" spans="1:5">
       <c r="A14" s="2" t="s">
         <v>32</v>
       </c>
@@ -751,7 +889,7 @@
         <v>33</v>
       </c>
       <c r="C14" s="2">
-        <f t="shared" si="1"/>
+        <f>50000000+ROW(A12)+1</f>
         <v>50000013</v>
       </c>
       <c r="D14" s="3" t="s">
@@ -761,7 +899,7 @@
         <v>4.0</v>
       </c>
     </row>
-    <row r="15">
+    <row r="15" spans="1:5">
       <c r="A15" s="2" t="s">
         <v>34</v>
       </c>
@@ -769,7 +907,7 @@
         <v>35</v>
       </c>
       <c r="C15" s="2">
-        <f t="shared" si="1"/>
+        <f>50000000+ROW(A13)+1</f>
         <v>50000014</v>
       </c>
       <c r="D15" s="3" t="s">
@@ -779,7 +917,7 @@
         <v>4.0</v>
       </c>
     </row>
-    <row r="16">
+    <row r="16" spans="1:5">
       <c r="A16" s="2" t="s">
         <v>36</v>
       </c>
@@ -787,7 +925,7 @@
         <v>37</v>
       </c>
       <c r="C16" s="2">
-        <f t="shared" si="1"/>
+        <f>50000000+ROW(A14)+1</f>
         <v>50000015</v>
       </c>
       <c r="D16" s="3" t="s">
@@ -797,7 +935,7 @@
         <v>4.0</v>
       </c>
     </row>
-    <row r="17">
+    <row r="17" spans="1:5">
       <c r="A17" s="2" t="s">
         <v>38</v>
       </c>
@@ -805,7 +943,7 @@
         <v>39</v>
       </c>
       <c r="C17" s="2">
-        <f t="shared" si="1"/>
+        <f>50000000+ROW(A15)+1</f>
         <v>50000016</v>
       </c>
       <c r="D17" s="3" t="s">
@@ -815,7 +953,7 @@
         <v>4.0</v>
       </c>
     </row>
-    <row r="18">
+    <row r="18" spans="1:5">
       <c r="A18" s="2" t="s">
         <v>40</v>
       </c>
@@ -823,7 +961,7 @@
         <v>41</v>
       </c>
       <c r="C18" s="2">
-        <f t="shared" si="1"/>
+        <f>50000000+ROW(A16)+1</f>
         <v>50000017</v>
       </c>
       <c r="D18" s="3" t="s">
@@ -833,7 +971,7 @@
         <v>4.0</v>
       </c>
     </row>
-    <row r="19">
+    <row r="19" spans="1:5">
       <c r="A19" s="2" t="s">
         <v>42</v>
       </c>
@@ -841,7 +979,7 @@
         <v>43</v>
       </c>
       <c r="C19" s="2">
-        <f t="shared" si="1"/>
+        <f>50000000+ROW(A17)+1</f>
         <v>50000018</v>
       </c>
       <c r="D19" s="3" t="s">
@@ -851,7 +989,7 @@
         <v>4.0</v>
       </c>
     </row>
-    <row r="20">
+    <row r="20" spans="1:5">
       <c r="A20" s="2" t="s">
         <v>44</v>
       </c>
@@ -859,7 +997,7 @@
         <v>45</v>
       </c>
       <c r="C20" s="2">
-        <f t="shared" si="1"/>
+        <f>50000000+ROW(A18)+1</f>
         <v>50000019</v>
       </c>
       <c r="D20" s="3" t="s">
@@ -869,7 +1007,7 @@
         <v>4.0</v>
       </c>
     </row>
-    <row r="21">
+    <row r="21" spans="1:5">
       <c r="A21" s="2" t="s">
         <v>46</v>
       </c>
@@ -877,7 +1015,7 @@
         <v>47</v>
       </c>
       <c r="C21" s="2">
-        <f t="shared" si="1"/>
+        <f>50000000+ROW(A19)+1</f>
         <v>50000020</v>
       </c>
       <c r="D21" s="3" t="s">
@@ -887,7 +1025,7 @@
         <v>2.0</v>
       </c>
     </row>
-    <row r="22">
+    <row r="22" spans="1:5">
       <c r="A22" s="2" t="s">
         <v>5</v>
       </c>
@@ -895,7 +1033,7 @@
         <v>48</v>
       </c>
       <c r="C22" s="2">
-        <f t="shared" si="1"/>
+        <f>50000000+ROW(A20)+1</f>
         <v>50000021</v>
       </c>
       <c r="D22" s="3" t="s">
@@ -905,7 +1043,7 @@
         <v>4.0</v>
       </c>
     </row>
-    <row r="23">
+    <row r="23" spans="1:5">
       <c r="A23" s="2" t="s">
         <v>8</v>
       </c>
@@ -913,7 +1051,7 @@
         <v>6</v>
       </c>
       <c r="C23" s="2">
-        <f t="shared" si="1"/>
+        <f>50000000+ROW(A21)+1</f>
         <v>50000022</v>
       </c>
       <c r="D23" s="3" t="s">
@@ -923,7 +1061,7 @@
         <v>4.0</v>
       </c>
     </row>
-    <row r="24">
+    <row r="24" spans="1:5">
       <c r="A24" s="2" t="s">
         <v>10</v>
       </c>
@@ -931,7 +1069,7 @@
         <v>9</v>
       </c>
       <c r="C24" s="2">
-        <f t="shared" si="1"/>
+        <f>50000000+ROW(A22)+1</f>
         <v>50000023</v>
       </c>
       <c r="D24" s="3" t="s">
@@ -941,7 +1079,7 @@
         <v>4.0</v>
       </c>
     </row>
-    <row r="25">
+    <row r="25" spans="1:5">
       <c r="A25" s="2" t="s">
         <v>13</v>
       </c>
@@ -949,7 +1087,7 @@
         <v>11</v>
       </c>
       <c r="C25" s="2">
-        <f t="shared" si="1"/>
+        <f>50000000+ROW(A23)+1</f>
         <v>50000024</v>
       </c>
       <c r="D25" s="3" t="s">
@@ -959,7 +1097,7 @@
         <v>4.0</v>
       </c>
     </row>
-    <row r="26">
+    <row r="26" spans="1:5">
       <c r="A26" s="2" t="s">
         <v>15</v>
       </c>
@@ -967,7 +1105,7 @@
         <v>14</v>
       </c>
       <c r="C26" s="2">
-        <f t="shared" si="1"/>
+        <f>50000000+ROW(A24)+1</f>
         <v>50000025</v>
       </c>
       <c r="D26" s="3" t="s">
@@ -977,7 +1115,7 @@
         <v>4.0</v>
       </c>
     </row>
-    <row r="27">
+    <row r="27" spans="1:5">
       <c r="A27" s="2" t="s">
         <v>17</v>
       </c>
@@ -985,7 +1123,7 @@
         <v>16</v>
       </c>
       <c r="C27" s="2">
-        <f t="shared" si="1"/>
+        <f>50000000+ROW(A25)+1</f>
         <v>50000026</v>
       </c>
       <c r="D27" s="3" t="s">
@@ -995,7 +1133,7 @@
         <v>2.0</v>
       </c>
     </row>
-    <row r="28">
+    <row r="28" spans="1:5">
       <c r="A28" s="2" t="s">
         <v>19</v>
       </c>
@@ -1003,7 +1141,7 @@
         <v>18</v>
       </c>
       <c r="C28" s="2">
-        <f t="shared" si="1"/>
+        <f>50000000+ROW(A26)+1</f>
         <v>50000027</v>
       </c>
       <c r="D28" s="3" t="s">
@@ -1013,7 +1151,7 @@
         <v>4.0</v>
       </c>
     </row>
-    <row r="29">
+    <row r="29" spans="1:5">
       <c r="A29" s="2" t="s">
         <v>21</v>
       </c>
@@ -1021,7 +1159,7 @@
         <v>20</v>
       </c>
       <c r="C29" s="2">
-        <f t="shared" si="1"/>
+        <f>50000000+ROW(A27)+1</f>
         <v>50000028</v>
       </c>
       <c r="D29" s="3" t="s">
@@ -1031,7 +1169,7 @@
         <v>4.0</v>
       </c>
     </row>
-    <row r="30">
+    <row r="30" spans="1:5">
       <c r="A30" s="2" t="s">
         <v>23</v>
       </c>
@@ -1039,7 +1177,7 @@
         <v>22</v>
       </c>
       <c r="C30" s="2">
-        <f t="shared" si="1"/>
+        <f>50000000+ROW(A28)+1</f>
         <v>50000029</v>
       </c>
       <c r="D30" s="3" t="s">
@@ -1049,7 +1187,7 @@
         <v>2.0</v>
       </c>
     </row>
-    <row r="31">
+    <row r="31" spans="1:5">
       <c r="A31" s="2" t="s">
         <v>25</v>
       </c>
@@ -1057,7 +1195,7 @@
         <v>24</v>
       </c>
       <c r="C31" s="2">
-        <f t="shared" si="1"/>
+        <f>50000000+ROW(A29)+1</f>
         <v>50000030</v>
       </c>
       <c r="D31" s="3" t="s">
@@ -1067,7 +1205,7 @@
         <v>4.0</v>
       </c>
     </row>
-    <row r="32">
+    <row r="32" spans="1:5">
       <c r="A32" s="2" t="s">
         <v>28</v>
       </c>
@@ -1075,7 +1213,7 @@
         <v>26</v>
       </c>
       <c r="C32" s="2">
-        <f t="shared" si="1"/>
+        <f>50000000+ROW(A30)+1</f>
         <v>50000031</v>
       </c>
       <c r="D32" s="3" t="s">
@@ -1085,7 +1223,7 @@
         <v>4.0</v>
       </c>
     </row>
-    <row r="33">
+    <row r="33" spans="1:5">
       <c r="A33" s="2" t="s">
         <v>30</v>
       </c>
@@ -1093,7 +1231,7 @@
         <v>29</v>
       </c>
       <c r="C33" s="2">
-        <f t="shared" si="1"/>
+        <f>50000000+ROW(A31)+1</f>
         <v>50000032</v>
       </c>
       <c r="D33" s="3" t="s">
@@ -1103,7 +1241,7 @@
         <v>4.0</v>
       </c>
     </row>
-    <row r="34">
+    <row r="34" spans="1:5">
       <c r="A34" s="2" t="s">
         <v>32</v>
       </c>
@@ -1111,7 +1249,7 @@
         <v>31</v>
       </c>
       <c r="C34" s="2">
-        <f t="shared" si="1"/>
+        <f>50000000+ROW(A32)+1</f>
         <v>50000033</v>
       </c>
       <c r="D34" s="3" t="s">
@@ -1121,7 +1259,7 @@
         <v>4.0</v>
       </c>
     </row>
-    <row r="35">
+    <row r="35" spans="1:5">
       <c r="A35" s="2" t="s">
         <v>34</v>
       </c>
@@ -1129,7 +1267,7 @@
         <v>33</v>
       </c>
       <c r="C35" s="2">
-        <f t="shared" si="1"/>
+        <f>50000000+ROW(A33)+1</f>
         <v>50000034</v>
       </c>
       <c r="D35" s="3" t="s">
@@ -1139,7 +1277,7 @@
         <v>2.0</v>
       </c>
     </row>
-    <row r="36">
+    <row r="36" spans="1:5">
       <c r="A36" s="2" t="s">
         <v>36</v>
       </c>
@@ -1147,7 +1285,7 @@
         <v>35</v>
       </c>
       <c r="C36" s="2">
-        <f t="shared" si="1"/>
+        <f>50000000+ROW(A34)+1</f>
         <v>50000035</v>
       </c>
       <c r="D36" s="3" t="s">
@@ -1157,7 +1295,7 @@
         <v>4.0</v>
       </c>
     </row>
-    <row r="37">
+    <row r="37" spans="1:5">
       <c r="A37" s="2" t="s">
         <v>38</v>
       </c>
@@ -1165,7 +1303,7 @@
         <v>37</v>
       </c>
       <c r="C37" s="2">
-        <f t="shared" si="1"/>
+        <f>50000000+ROW(A35)+1</f>
         <v>50000036</v>
       </c>
       <c r="D37" s="3" t="s">
@@ -1175,7 +1313,7 @@
         <v>4.0</v>
       </c>
     </row>
-    <row r="38">
+    <row r="38" spans="1:5">
       <c r="A38" s="2" t="s">
         <v>40</v>
       </c>
@@ -1183,7 +1321,7 @@
         <v>39</v>
       </c>
       <c r="C38" s="2">
-        <f t="shared" si="1"/>
+        <f>50000000+ROW(A36)+1</f>
         <v>50000037</v>
       </c>
       <c r="D38" s="3" t="s">
@@ -1193,7 +1331,7 @@
         <v>4.0</v>
       </c>
     </row>
-    <row r="39">
+    <row r="39" spans="1:5">
       <c r="A39" s="2" t="s">
         <v>42</v>
       </c>
@@ -1201,7 +1339,7 @@
         <v>41</v>
       </c>
       <c r="C39" s="2">
-        <f t="shared" si="1"/>
+        <f>50000000+ROW(A37)+1</f>
         <v>50000038</v>
       </c>
       <c r="D39" s="5" t="s">
@@ -1211,7 +1349,7 @@
         <v>4.0</v>
       </c>
     </row>
-    <row r="40">
+    <row r="40" spans="1:5">
       <c r="A40" s="2" t="s">
         <v>44</v>
       </c>
@@ -1219,7 +1357,7 @@
         <v>43</v>
       </c>
       <c r="C40" s="2">
-        <f t="shared" si="1"/>
+        <f>50000000+ROW(A38)+1</f>
         <v>50000039</v>
       </c>
       <c r="D40" s="3" t="s">
@@ -1229,7 +1367,7 @@
         <v>4.0</v>
       </c>
     </row>
-    <row r="41">
+    <row r="41" spans="1:5">
       <c r="A41" s="2" t="s">
         <v>46</v>
       </c>
@@ -1237,7 +1375,7 @@
         <v>45</v>
       </c>
       <c r="C41" s="2">
-        <f t="shared" si="1"/>
+        <f>50000000+ROW(A39)+1</f>
         <v>50000040</v>
       </c>
       <c r="D41" s="3" t="s">
@@ -1247,7 +1385,7 @@
         <v>4.0</v>
       </c>
     </row>
-    <row r="42">
+    <row r="42" spans="1:5">
       <c r="A42" s="2" t="s">
         <v>5</v>
       </c>
@@ -1255,7 +1393,7 @@
         <v>47</v>
       </c>
       <c r="C42" s="2">
-        <f t="shared" si="1"/>
+        <f>50000000+ROW(A40)+1</f>
         <v>50000041</v>
       </c>
       <c r="D42" s="3" t="s">
@@ -1265,15 +1403,15 @@
         <v>4.0</v>
       </c>
     </row>
-    <row r="43">
+    <row r="43" spans="1:5">
       <c r="A43" s="2" t="s">
-        <v>8</v>
+        <v>49</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>6</v>
+        <v>50</v>
       </c>
       <c r="C43" s="2">
-        <f t="shared" si="1"/>
+        <f>50000000+ROW(A41)+1</f>
         <v>50000042</v>
       </c>
       <c r="D43" s="3" t="s">
@@ -1283,15 +1421,15 @@
         <v>4.0</v>
       </c>
     </row>
-    <row r="44">
+    <row r="44" spans="1:5">
       <c r="A44" s="2" t="s">
-        <v>10</v>
+        <v>51</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>9</v>
+        <v>52</v>
       </c>
       <c r="C44" s="2">
-        <f t="shared" si="1"/>
+        <f>50000000+ROW(A42)+1</f>
         <v>50000043</v>
       </c>
       <c r="D44" s="3" t="s">
@@ -1301,15 +1439,15 @@
         <v>4.0</v>
       </c>
     </row>
-    <row r="45">
+    <row r="45" spans="1:5">
       <c r="A45" s="2" t="s">
-        <v>13</v>
+        <v>53</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>11</v>
+        <v>54</v>
       </c>
       <c r="C45" s="2">
-        <f t="shared" si="1"/>
+        <f>50000000+ROW(A43)+1</f>
         <v>50000044</v>
       </c>
       <c r="D45" s="3" t="s">
@@ -1319,15 +1457,15 @@
         <v>3.0</v>
       </c>
     </row>
-    <row r="46">
+    <row r="46" spans="1:5">
       <c r="A46" s="2" t="s">
-        <v>15</v>
+        <v>55</v>
       </c>
       <c r="B46" s="2" t="s">
-        <v>14</v>
+        <v>56</v>
       </c>
       <c r="C46" s="2">
-        <f t="shared" si="1"/>
+        <f>50000000+ROW(A44)+1</f>
         <v>50000045</v>
       </c>
       <c r="D46" s="3" t="s">
@@ -1337,15 +1475,15 @@
         <v>4.0</v>
       </c>
     </row>
-    <row r="47">
+    <row r="47" spans="1:5">
       <c r="A47" s="2" t="s">
-        <v>17</v>
+        <v>57</v>
       </c>
       <c r="B47" s="2" t="s">
-        <v>16</v>
+        <v>58</v>
       </c>
       <c r="C47" s="2">
-        <f t="shared" si="1"/>
+        <f>50000000+ROW(A45)+1</f>
         <v>50000046</v>
       </c>
       <c r="D47" s="3" t="s">
@@ -1355,15 +1493,15 @@
         <v>4.0</v>
       </c>
     </row>
-    <row r="48">
+    <row r="48" spans="1:5">
       <c r="A48" s="2" t="s">
-        <v>19</v>
+        <v>59</v>
       </c>
       <c r="B48" s="2" t="s">
-        <v>18</v>
+        <v>60</v>
       </c>
       <c r="C48" s="2">
-        <f t="shared" si="1"/>
+        <f>50000000+ROW(A46)+1</f>
         <v>50000047</v>
       </c>
       <c r="D48" s="3" t="s">
@@ -1373,15 +1511,15 @@
         <v>4.0</v>
       </c>
     </row>
-    <row r="49">
+    <row r="49" spans="1:5">
       <c r="A49" s="2" t="s">
-        <v>21</v>
+        <v>61</v>
       </c>
       <c r="B49" s="2" t="s">
-        <v>20</v>
+        <v>62</v>
       </c>
       <c r="C49" s="2">
-        <f t="shared" si="1"/>
+        <f>50000000+ROW(A47)+1</f>
         <v>50000048</v>
       </c>
       <c r="D49" s="3" t="s">
@@ -1391,15 +1529,15 @@
         <v>2.0</v>
       </c>
     </row>
-    <row r="50">
+    <row r="50" spans="1:5">
       <c r="A50" s="2" t="s">
-        <v>23</v>
+        <v>63</v>
       </c>
       <c r="B50" s="2" t="s">
-        <v>22</v>
+        <v>64</v>
       </c>
       <c r="C50" s="2">
-        <f t="shared" si="1"/>
+        <f>50000000+ROW(A48)+1</f>
         <v>50000049</v>
       </c>
       <c r="D50" s="5" t="s">
@@ -1409,15 +1547,15 @@
         <v>2.0</v>
       </c>
     </row>
-    <row r="51">
+    <row r="51" spans="1:5">
       <c r="A51" s="2" t="s">
-        <v>25</v>
+        <v>65</v>
       </c>
       <c r="B51" s="2" t="s">
-        <v>24</v>
+        <v>66</v>
       </c>
       <c r="C51" s="2">
-        <f t="shared" si="1"/>
+        <f>50000000+ROW(A49)+1</f>
         <v>50000050</v>
       </c>
       <c r="D51" s="5" t="s">
@@ -1427,15 +1565,15 @@
         <v>4.0</v>
       </c>
     </row>
-    <row r="52">
+    <row r="52" spans="1:5">
       <c r="A52" s="2" t="s">
-        <v>28</v>
+        <v>67</v>
       </c>
       <c r="B52" s="2" t="s">
-        <v>26</v>
+        <v>68</v>
       </c>
       <c r="C52" s="2">
-        <f t="shared" si="1"/>
+        <f>50000000+ROW(A50)+1</f>
         <v>50000051</v>
       </c>
       <c r="D52" s="3" t="s">
@@ -1445,15 +1583,15 @@
         <v>4.0</v>
       </c>
     </row>
-    <row r="53">
+    <row r="53" spans="1:5">
       <c r="A53" s="2" t="s">
-        <v>30</v>
+        <v>69</v>
       </c>
       <c r="B53" s="2" t="s">
-        <v>29</v>
+        <v>70</v>
       </c>
       <c r="C53" s="2">
-        <f t="shared" si="1"/>
+        <f>50000000+ROW(A51)+1</f>
         <v>50000052</v>
       </c>
       <c r="D53" s="3" t="s">
@@ -1463,15 +1601,15 @@
         <v>3.0</v>
       </c>
     </row>
-    <row r="54">
+    <row r="54" spans="1:5">
       <c r="A54" s="2" t="s">
-        <v>32</v>
+        <v>71</v>
       </c>
       <c r="B54" s="2" t="s">
-        <v>31</v>
+        <v>72</v>
       </c>
       <c r="C54" s="2">
-        <f t="shared" si="1"/>
+        <f>50000000+ROW(A52)+1</f>
         <v>50000053</v>
       </c>
       <c r="D54" s="3" t="s">
@@ -1481,15 +1619,15 @@
         <v>3.0</v>
       </c>
     </row>
-    <row r="55">
+    <row r="55" spans="1:5">
       <c r="A55" s="2" t="s">
-        <v>34</v>
+        <v>73</v>
       </c>
       <c r="B55" s="2" t="s">
-        <v>33</v>
+        <v>74</v>
       </c>
       <c r="C55" s="2">
-        <f t="shared" si="1"/>
+        <f>50000000+ROW(A53)+1</f>
         <v>50000054</v>
       </c>
       <c r="D55" s="3" t="s">
@@ -1499,15 +1637,15 @@
         <v>2.0</v>
       </c>
     </row>
-    <row r="56">
+    <row r="56" spans="1:5">
       <c r="A56" s="2" t="s">
-        <v>36</v>
+        <v>75</v>
       </c>
       <c r="B56" s="2" t="s">
-        <v>35</v>
+        <v>76</v>
       </c>
       <c r="C56" s="2">
-        <f t="shared" si="1"/>
+        <f>50000000+ROW(A54)+1</f>
         <v>50000055</v>
       </c>
       <c r="D56" s="3" t="s">
@@ -1517,15 +1655,15 @@
         <v>4.0</v>
       </c>
     </row>
-    <row r="57">
+    <row r="57" spans="1:5">
       <c r="A57" s="2" t="s">
-        <v>38</v>
+        <v>77</v>
       </c>
       <c r="B57" s="2" t="s">
-        <v>37</v>
+        <v>78</v>
       </c>
       <c r="C57" s="2">
-        <f t="shared" si="1"/>
+        <f>50000000+ROW(A55)+1</f>
         <v>50000056</v>
       </c>
       <c r="D57" s="5" t="s">
@@ -1535,15 +1673,15 @@
         <v>4.0</v>
       </c>
     </row>
-    <row r="58">
+    <row r="58" spans="1:5">
       <c r="A58" s="2" t="s">
-        <v>40</v>
+        <v>79</v>
       </c>
       <c r="B58" s="2" t="s">
-        <v>39</v>
+        <v>80</v>
       </c>
       <c r="C58" s="2">
-        <f t="shared" si="1"/>
+        <f>50000000+ROW(A56)+1</f>
         <v>50000057</v>
       </c>
       <c r="D58" s="3" t="s">
@@ -1553,15 +1691,15 @@
         <v>4.0</v>
       </c>
     </row>
-    <row r="59">
+    <row r="59" spans="1:5">
       <c r="A59" s="2" t="s">
-        <v>42</v>
+        <v>81</v>
       </c>
       <c r="B59" s="2" t="s">
-        <v>41</v>
+        <v>82</v>
       </c>
       <c r="C59" s="2">
-        <f t="shared" si="1"/>
+        <f>50000000+ROW(A57)+1</f>
         <v>50000058</v>
       </c>
       <c r="D59" s="3" t="s">
@@ -1571,15 +1709,15 @@
         <v>2.0</v>
       </c>
     </row>
-    <row r="60">
+    <row r="60" spans="1:5">
       <c r="A60" s="2" t="s">
-        <v>44</v>
+        <v>83</v>
       </c>
       <c r="B60" s="2" t="s">
-        <v>43</v>
+        <v>84</v>
       </c>
       <c r="C60" s="2">
-        <f t="shared" si="1"/>
+        <f>50000000+ROW(A58)+1</f>
         <v>50000059</v>
       </c>
       <c r="D60" s="3" t="s">
@@ -1589,15 +1727,15 @@
         <v>4.0</v>
       </c>
     </row>
-    <row r="61">
+    <row r="61" spans="1:5">
       <c r="A61" s="2" t="s">
-        <v>46</v>
+        <v>85</v>
       </c>
       <c r="B61" s="2" t="s">
-        <v>45</v>
+        <v>86</v>
       </c>
       <c r="C61" s="2">
-        <f t="shared" si="1"/>
+        <f>50000000+ROW(A59)+1</f>
         <v>50000060</v>
       </c>
       <c r="D61" s="3" t="s">
@@ -1608,9 +1746,20 @@
       </c>
     </row>
   </sheetData>
+  <printOptions gridLines="false" gridLinesSet="true"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="1" orientation="default" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver"/>
+  <headerFooter differentOddEven="false" differentFirst="false" scaleWithDoc="true" alignWithMargins="true">
+    <oddHeader/>
+    <oddFooter/>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
   <drawing r:id="rId1"/>
   <tableParts count="1">
-    <tablePart r:id="rId3"/>
+    <tablePart r:id="rId_table_1"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix: alinear nombres con el género registrado en el padrón de ejemplo
El equilibrio de género ya se aplicaba por género registrado (columna
Género), pero el padrón de prueba tenía nombres cruzados (ej. "Juan
Gómez" registrado como mujer), lo que hacía parecer que los titulares
eran casi todos varones. Se renombraron 24 filas para que el nombre
coincida con el género registrado, sin tocar género, DNI ni tipo.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/example-ppc.xlsx
+++ b/example-ppc.xlsx
@@ -43,130 +43,139 @@
     <t>M</t>
   </si>
   <si>
+    <t>Gómez</t>
+  </si>
+  <si>
     <t>Juan</t>
   </si>
   <si>
-    <t>Gómez</t>
+    <t>López</t>
+  </si>
+  <si>
+    <t>V</t>
+  </si>
+  <si>
+    <t>Pedro</t>
+  </si>
+  <si>
+    <t>Martínez</t>
+  </si>
+  <si>
+    <t>Rodríguez</t>
+  </si>
+  <si>
+    <t>Martín</t>
+  </si>
+  <si>
+    <t>Sánchez</t>
+  </si>
+  <si>
+    <t>Sofía</t>
+  </si>
+  <si>
+    <t>Ramírez</t>
   </si>
   <si>
     <t>María</t>
   </si>
   <si>
-    <t>López</t>
-  </si>
-  <si>
-    <t>V</t>
-  </si>
-  <si>
-    <t>Pedro</t>
-  </si>
-  <si>
-    <t>Martínez</t>
+    <t>Torres</t>
+  </si>
+  <si>
+    <t>Herrera</t>
+  </si>
+  <si>
+    <t>Nicolás</t>
+  </si>
+  <si>
+    <t>Benítez</t>
+  </si>
+  <si>
+    <t>O</t>
+  </si>
+  <si>
+    <t>Diego</t>
+  </si>
+  <si>
+    <t>Pérez</t>
   </si>
   <si>
     <t>Lucía</t>
   </si>
   <si>
-    <t>Rodríguez</t>
-  </si>
-  <si>
-    <t>Martín</t>
-  </si>
-  <si>
-    <t>Sánchez</t>
-  </si>
-  <si>
-    <t>Sofía</t>
-  </si>
-  <si>
-    <t>Ramírez</t>
-  </si>
-  <si>
-    <t>Diego</t>
-  </si>
-  <si>
-    <t>Torres</t>
+    <t>Alvarez</t>
+  </si>
+  <si>
+    <t>Romero</t>
+  </si>
+  <si>
+    <t>Tomás</t>
+  </si>
+  <si>
+    <t>Silva</t>
+  </si>
+  <si>
+    <t>Franco</t>
+  </si>
+  <si>
+    <t>Ruiz</t>
+  </si>
+  <si>
+    <t>Lucas</t>
+  </si>
+  <si>
+    <t>Acosta</t>
+  </si>
+  <si>
+    <t>Castro</t>
+  </si>
+  <si>
+    <t>Medina</t>
+  </si>
+  <si>
+    <t>Molina</t>
   </si>
   <si>
     <t>Valentina</t>
   </si>
   <si>
-    <t>Herrera</t>
-  </si>
-  <si>
-    <t>Nicolás</t>
-  </si>
-  <si>
-    <t>Benítez</t>
-  </si>
-  <si>
-    <t>O</t>
+    <t>Vega</t>
+  </si>
+  <si>
+    <t>Rodriguez</t>
   </si>
   <si>
     <t>Camila</t>
   </si>
   <si>
-    <t>Pérez</t>
-  </si>
-  <si>
-    <t>Franco</t>
-  </si>
-  <si>
-    <t>Alvarez</t>
+    <t>Mateo</t>
   </si>
   <si>
     <t>Julieta</t>
   </si>
   <si>
-    <t>Romero</t>
-  </si>
-  <si>
-    <t>Tomás</t>
-  </si>
-  <si>
-    <t>Silva</t>
-  </si>
-  <si>
     <t>Agustina</t>
   </si>
   <si>
-    <t>Ruiz</t>
-  </si>
-  <si>
-    <t>Lucas</t>
-  </si>
-  <si>
-    <t>Acosta</t>
+    <t>Joaquín</t>
   </si>
   <si>
     <t>Carla</t>
   </si>
   <si>
-    <t>Castro</t>
-  </si>
-  <si>
-    <t>Mateo</t>
-  </si>
-  <si>
-    <t>Medina</t>
+    <t>Ramiro</t>
   </si>
   <si>
     <t>Florencia</t>
   </si>
   <si>
-    <t>Molina</t>
-  </si>
-  <si>
-    <t>Joaquín</t>
-  </si>
-  <si>
-    <t>Vega</t>
-  </si>
-  <si>
-    <t>Rodriguez</t>
-  </si>
-  <si>
-    <t>Ramiro</t>
+    <t>Esteban</t>
+  </si>
+  <si>
+    <t>Daniela</t>
+  </si>
+  <si>
+    <t>Gonzalo</t>
   </si>
   <si>
     <t>Ledesma</t>
@@ -178,9 +187,6 @@
     <t>Giménez</t>
   </si>
   <si>
-    <t>Esteban</t>
-  </si>
-  <si>
     <t>Núñez</t>
   </si>
   <si>
@@ -190,9 +196,6 @@
     <t>Cabrera</t>
   </si>
   <si>
-    <t>Gonzalo</t>
-  </si>
-  <si>
     <t>Duarte</t>
   </si>
   <si>
@@ -218,9 +221,6 @@
   </si>
   <si>
     <t>Aguirre</t>
-  </si>
-  <si>
-    <t>Daniela</t>
   </si>
   <si>
     <t>Ferreyra</t>
@@ -685,10 +685,10 @@
     </row>
     <row r="3" spans="1:5">
       <c r="A3" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B3" s="2" t="s">
         <v>8</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>9</v>
       </c>
       <c r="C3" s="2">
         <f>50000000+ROW(A1)+1</f>
@@ -703,17 +703,17 @@
     </row>
     <row r="4" spans="1:5">
       <c r="A4" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4" s="2" t="s">
         <v>10</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>11</v>
       </c>
       <c r="C4" s="2">
         <f>50000000+ROW(A2)+1</f>
         <v>50000003</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E4" s="2">
         <v>4.0</v>
@@ -721,17 +721,17 @@
     </row>
     <row r="5" spans="1:5">
       <c r="A5" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B5" s="2" t="s">
         <v>13</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>14</v>
       </c>
       <c r="C5" s="2">
         <f>50000000+ROW(A3)+1</f>
         <v>50000004</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E5" s="4">
         <v>3.0</v>
@@ -739,17 +739,17 @@
     </row>
     <row r="6" spans="1:5">
       <c r="A6" s="2" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="C6" s="2">
         <f>50000000+ROW(A4)+1</f>
         <v>50000005</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E6" s="4">
         <v>3.0</v>
@@ -757,17 +757,17 @@
     </row>
     <row r="7" spans="1:5">
       <c r="A7" s="2" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="C7" s="2">
         <f>50000000+ROW(A5)+1</f>
         <v>50000006</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E7" s="4">
         <v>4.0</v>
@@ -775,10 +775,10 @@
     </row>
     <row r="8" spans="1:5">
       <c r="A8" s="2" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="C8" s="2">
         <f>50000000+ROW(A6)+1</f>
@@ -793,10 +793,10 @@
     </row>
     <row r="9" spans="1:5">
       <c r="A9" s="2" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="C9" s="2">
         <f>50000000+ROW(A7)+1</f>
@@ -811,17 +811,17 @@
     </row>
     <row r="10" spans="1:5">
       <c r="A10" s="2" t="s">
-        <v>23</v>
+        <v>15</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="C10" s="2">
         <f>50000000+ROW(A8)+1</f>
         <v>50000009</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E10" s="4">
         <v>4.0</v>
@@ -829,17 +829,17 @@
     </row>
     <row r="11" spans="1:5">
       <c r="A11" s="2" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="C11" s="2">
         <f>50000000+ROW(A9)+1</f>
         <v>50000010</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="E11" s="4">
         <v>3.0</v>
@@ -847,17 +847,17 @@
     </row>
     <row r="12" spans="1:5">
       <c r="A12" s="2" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="C12" s="2">
         <f>50000000+ROW(A10)+1</f>
         <v>50000011</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E12" s="4">
         <v>3.0</v>
@@ -865,10 +865,10 @@
     </row>
     <row r="13" spans="1:5">
       <c r="A13" s="2" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="C13" s="2">
         <f>50000000+ROW(A11)+1</f>
@@ -883,17 +883,17 @@
     </row>
     <row r="14" spans="1:5">
       <c r="A14" s="2" t="s">
-        <v>32</v>
+        <v>22</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="C14" s="2">
         <f>50000000+ROW(A12)+1</f>
         <v>50000013</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E14" s="4">
         <v>4.0</v>
@@ -901,17 +901,17 @@
     </row>
     <row r="15" spans="1:5">
       <c r="A15" s="2" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="C15" s="2">
         <f>50000000+ROW(A13)+1</f>
         <v>50000014</v>
       </c>
       <c r="D15" s="3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E15" s="4">
         <v>4.0</v>
@@ -919,17 +919,17 @@
     </row>
     <row r="16" spans="1:5">
       <c r="A16" s="2" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="C16" s="2">
         <f>50000000+ROW(A14)+1</f>
         <v>50000015</v>
       </c>
       <c r="D16" s="3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E16" s="4">
         <v>4.0</v>
@@ -937,17 +937,17 @@
     </row>
     <row r="17" spans="1:5">
       <c r="A17" s="2" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="C17" s="2">
         <f>50000000+ROW(A15)+1</f>
         <v>50000016</v>
       </c>
       <c r="D17" s="3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E17" s="4">
         <v>4.0</v>
@@ -955,17 +955,17 @@
     </row>
     <row r="18" spans="1:5">
       <c r="A18" s="2" t="s">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="C18" s="2">
         <f>50000000+ROW(A16)+1</f>
         <v>50000017</v>
       </c>
       <c r="D18" s="3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E18" s="4">
         <v>4.0</v>
@@ -973,10 +973,10 @@
     </row>
     <row r="19" spans="1:5">
       <c r="A19" s="2" t="s">
-        <v>42</v>
+        <v>17</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>43</v>
+        <v>37</v>
       </c>
       <c r="C19" s="2">
         <f>50000000+ROW(A17)+1</f>
@@ -991,17 +991,17 @@
     </row>
     <row r="20" spans="1:5">
       <c r="A20" s="2" t="s">
-        <v>44</v>
+        <v>34</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>45</v>
+        <v>38</v>
       </c>
       <c r="C20" s="2">
         <f>50000000+ROW(A18)+1</f>
         <v>50000019</v>
       </c>
       <c r="D20" s="3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E20" s="4">
         <v>4.0</v>
@@ -1009,10 +1009,10 @@
     </row>
     <row r="21" spans="1:5">
       <c r="A21" s="2" t="s">
-        <v>46</v>
+        <v>39</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>47</v>
+        <v>40</v>
       </c>
       <c r="C21" s="2">
         <f>50000000+ROW(A19)+1</f>
@@ -1030,7 +1030,7 @@
         <v>5</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>48</v>
+        <v>41</v>
       </c>
       <c r="C22" s="2">
         <f>50000000+ROW(A20)+1</f>
@@ -1045,7 +1045,7 @@
     </row>
     <row r="23" spans="1:5">
       <c r="A23" s="2" t="s">
-        <v>8</v>
+        <v>42</v>
       </c>
       <c r="B23" s="2" t="s">
         <v>6</v>
@@ -1063,10 +1063,10 @@
     </row>
     <row r="24" spans="1:5">
       <c r="A24" s="2" t="s">
-        <v>10</v>
+        <v>19</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C24" s="2">
         <f>50000000+ROW(A22)+1</f>
@@ -1081,17 +1081,17 @@
     </row>
     <row r="25" spans="1:5">
       <c r="A25" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C25" s="2">
         <f>50000000+ROW(A23)+1</f>
         <v>50000024</v>
       </c>
       <c r="D25" s="3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E25" s="4">
         <v>4.0</v>
@@ -1099,17 +1099,17 @@
     </row>
     <row r="26" spans="1:5">
       <c r="A26" s="2" t="s">
-        <v>15</v>
+        <v>43</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C26" s="2">
         <f>50000000+ROW(A24)+1</f>
         <v>50000025</v>
       </c>
       <c r="D26" s="3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E26" s="4">
         <v>4.0</v>
@@ -1117,17 +1117,17 @@
     </row>
     <row r="27" spans="1:5">
       <c r="A27" s="2" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="C27" s="2">
         <f>50000000+ROW(A25)+1</f>
         <v>50000026</v>
       </c>
       <c r="D27" s="3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E27" s="4">
         <v>2.0</v>
@@ -1135,10 +1135,10 @@
     </row>
     <row r="28" spans="1:5">
       <c r="A28" s="2" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="C28" s="2">
         <f>50000000+ROW(A26)+1</f>
@@ -1153,17 +1153,17 @@
     </row>
     <row r="29" spans="1:5">
       <c r="A29" s="2" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="C29" s="2">
         <f>50000000+ROW(A27)+1</f>
         <v>50000028</v>
       </c>
       <c r="D29" s="3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E29" s="4">
         <v>4.0</v>
@@ -1171,10 +1171,10 @@
     </row>
     <row r="30" spans="1:5">
       <c r="A30" s="2" t="s">
-        <v>23</v>
+        <v>39</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="C30" s="2">
         <f>50000000+ROW(A28)+1</f>
@@ -1189,10 +1189,10 @@
     </row>
     <row r="31" spans="1:5">
       <c r="A31" s="2" t="s">
-        <v>25</v>
+        <v>44</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="C31" s="2">
         <f>50000000+ROW(A29)+1</f>
@@ -1207,10 +1207,10 @@
     </row>
     <row r="32" spans="1:5">
       <c r="A32" s="2" t="s">
-        <v>28</v>
+        <v>42</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="C32" s="2">
         <f>50000000+ROW(A30)+1</f>
@@ -1225,10 +1225,10 @@
     </row>
     <row r="33" spans="1:5">
       <c r="A33" s="2" t="s">
-        <v>30</v>
+        <v>45</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="C33" s="2">
         <f>50000000+ROW(A31)+1</f>
@@ -1243,17 +1243,17 @@
     </row>
     <row r="34" spans="1:5">
       <c r="A34" s="2" t="s">
-        <v>32</v>
+        <v>46</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="C34" s="2">
         <f>50000000+ROW(A32)+1</f>
         <v>50000033</v>
       </c>
       <c r="D34" s="3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E34" s="4">
         <v>4.0</v>
@@ -1261,10 +1261,10 @@
     </row>
     <row r="35" spans="1:5">
       <c r="A35" s="2" t="s">
-        <v>34</v>
+        <v>47</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="C35" s="2">
         <f>50000000+ROW(A33)+1</f>
@@ -1279,17 +1279,17 @@
     </row>
     <row r="36" spans="1:5">
       <c r="A36" s="2" t="s">
-        <v>36</v>
+        <v>48</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="C36" s="2">
         <f>50000000+ROW(A34)+1</f>
         <v>50000035</v>
       </c>
       <c r="D36" s="3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E36" s="4">
         <v>4.0</v>
@@ -1297,10 +1297,10 @@
     </row>
     <row r="37" spans="1:5">
       <c r="A37" s="2" t="s">
-        <v>38</v>
+        <v>49</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="C37" s="2">
         <f>50000000+ROW(A35)+1</f>
@@ -1315,17 +1315,17 @@
     </row>
     <row r="38" spans="1:5">
       <c r="A38" s="2" t="s">
-        <v>40</v>
+        <v>50</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="C38" s="2">
         <f>50000000+ROW(A36)+1</f>
         <v>50000037</v>
       </c>
       <c r="D38" s="3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E38" s="4">
         <v>4.0</v>
@@ -1333,17 +1333,17 @@
     </row>
     <row r="39" spans="1:5">
       <c r="A39" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="C39" s="2">
         <f>50000000+ROW(A37)+1</f>
         <v>50000038</v>
       </c>
       <c r="D39" s="5" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="E39" s="4">
         <v>4.0</v>
@@ -1351,10 +1351,10 @@
     </row>
     <row r="40" spans="1:5">
       <c r="A40" s="2" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>43</v>
+        <v>37</v>
       </c>
       <c r="C40" s="2">
         <f>50000000+ROW(A38)+1</f>
@@ -1369,10 +1369,10 @@
     </row>
     <row r="41" spans="1:5">
       <c r="A41" s="2" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>45</v>
+        <v>38</v>
       </c>
       <c r="C41" s="2">
         <f>50000000+ROW(A39)+1</f>
@@ -1387,17 +1387,17 @@
     </row>
     <row r="42" spans="1:5">
       <c r="A42" s="2" t="s">
-        <v>5</v>
+        <v>52</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>47</v>
+        <v>40</v>
       </c>
       <c r="C42" s="2">
         <f>50000000+ROW(A40)+1</f>
         <v>50000041</v>
       </c>
       <c r="D42" s="3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E42" s="4">
         <v>4.0</v>
@@ -1405,17 +1405,17 @@
     </row>
     <row r="43" spans="1:5">
       <c r="A43" s="2" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="C43" s="2">
         <f>50000000+ROW(A41)+1</f>
         <v>50000042</v>
       </c>
       <c r="D43" s="3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E43" s="4">
         <v>4.0</v>
@@ -1423,10 +1423,10 @@
     </row>
     <row r="44" spans="1:5">
       <c r="A44" s="2" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="C44" s="2">
         <f>50000000+ROW(A42)+1</f>
@@ -1441,17 +1441,17 @@
     </row>
     <row r="45" spans="1:5">
       <c r="A45" s="2" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="C45" s="2">
         <f>50000000+ROW(A43)+1</f>
         <v>50000044</v>
       </c>
       <c r="D45" s="3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E45" s="4">
         <v>3.0</v>
@@ -1459,10 +1459,10 @@
     </row>
     <row r="46" spans="1:5">
       <c r="A46" s="2" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="B46" s="2" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C46" s="2">
         <f>50000000+ROW(A44)+1</f>
@@ -1477,17 +1477,17 @@
     </row>
     <row r="47" spans="1:5">
       <c r="A47" s="2" t="s">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="B47" s="2" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C47" s="2">
         <f>50000000+ROW(A45)+1</f>
         <v>50000046</v>
       </c>
       <c r="D47" s="3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E47" s="4">
         <v>4.0</v>
@@ -1495,10 +1495,10 @@
     </row>
     <row r="48" spans="1:5">
       <c r="A48" s="2" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B48" s="2" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C48" s="2">
         <f>50000000+ROW(A46)+1</f>
@@ -1513,17 +1513,17 @@
     </row>
     <row r="49" spans="1:5">
       <c r="A49" s="2" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B49" s="2" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C49" s="2">
         <f>50000000+ROW(A47)+1</f>
         <v>50000048</v>
       </c>
       <c r="D49" s="3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E49" s="4">
         <v>2.0</v>
@@ -1531,10 +1531,10 @@
     </row>
     <row r="50" spans="1:5">
       <c r="A50" s="2" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B50" s="2" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C50" s="2">
         <f>50000000+ROW(A48)+1</f>
@@ -1549,17 +1549,17 @@
     </row>
     <row r="51" spans="1:5">
       <c r="A51" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B51" s="2" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C51" s="2">
         <f>50000000+ROW(A49)+1</f>
         <v>50000050</v>
       </c>
       <c r="D51" s="5" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="E51" s="4">
         <v>4.0</v>
@@ -1567,7 +1567,7 @@
     </row>
     <row r="52" spans="1:5">
       <c r="A52" s="2" t="s">
-        <v>67</v>
+        <v>51</v>
       </c>
       <c r="B52" s="2" t="s">
         <v>68</v>
@@ -1613,7 +1613,7 @@
         <v>50000053</v>
       </c>
       <c r="D54" s="3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E54" s="4">
         <v>3.0</v>
@@ -1631,7 +1631,7 @@
         <v>50000054</v>
       </c>
       <c r="D55" s="3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E55" s="4">
         <v>2.0</v>
@@ -1667,7 +1667,7 @@
         <v>50000056</v>
       </c>
       <c r="D57" s="5" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E57" s="4">
         <v>4.0</v>
@@ -1703,7 +1703,7 @@
         <v>50000058</v>
       </c>
       <c r="D59" s="3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E59" s="6">
         <v>2.0</v>
@@ -1721,7 +1721,7 @@
         <v>50000059</v>
       </c>
       <c r="D60" s="3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E60" s="6">
         <v>4.0</v>

</xml_diff>